<commit_message>
Opdateret IDOART skabelon og oploadet første draft af fælles vejledermøde
</commit_message>
<xml_diff>
--- a/docs/Fonde_2025.xlsx
+++ b/docs/Fonde_2025.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\R_document\phd\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D092ED1F-F9CC-4FE2-901C-DD1CE3602C25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B67C589-188F-4AAB-9990-BC99B102D3CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="56">
   <si>
     <t>Diabetesforeningen</t>
   </si>
@@ -186,6 +186,15 @@
   </si>
   <si>
     <t>40.000 - 100.000 kr.</t>
+  </si>
+  <si>
+    <t>DFF klinisk forskning</t>
+  </si>
+  <si>
+    <t>Start juni</t>
+  </si>
+  <si>
+    <t>Det aftal</t>
   </si>
 </sst>
 </file>
@@ -863,8 +872,15 @@
       </c>
     </row>
     <row r="14" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="E14" s="17"/>
-      <c r="F14" s="6"/>
+      <c r="A14" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="E14" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">

</xml_diff>